<commit_message>
Fixed file to update fuel price
Fixed file to update fuel price
</commit_message>
<xml_diff>
--- a/SuppXLS/Scen_SYS_FossilFuel_Update_DC.xlsx
+++ b/SuppXLS/Scen_SYS_FossilFuel_Update_DC.xlsx
@@ -8,13 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nuigalwayie-my.sharepoint.com/personal/d_cawley10_universityofgalway_ie/Documents/5th Year/RM3_Thesis_DataCentre_Hydrogen_Dermot/07_Data/times-ireland-model/SuppXLS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="19" documentId="11_F25DC773A252ABDACC10485FB99B509C5BDE58E6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A919648C-D243-429A-9101-7634B01FAF8A}"/>
+  <xr:revisionPtr revIDLastSave="32" documentId="11_F25DC773A252ABDACC10485FB99B509C5BDE58E6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D1F8B1B7-C5CB-4BF1-A889-72EAFE5FC016}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="3922" yWindow="3922" windowWidth="15390" windowHeight="9443" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="20715" windowHeight="13155" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <externalReferences>
+    <externalReference r:id="rId2"/>
+  </externalReferences>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -36,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="10">
   <si>
     <t>TimeSlice</t>
   </si>
@@ -47,12 +50,12 @@
     <t>Attribute</t>
   </si>
   <si>
+    <t>AllRegions</t>
+  </si>
+  <si>
     <t>IRE_PRICE</t>
   </si>
   <si>
-    <t>AllRegionsCSAT_CN</t>
-  </si>
-  <si>
     <t>Pset_PN</t>
   </si>
   <si>
@@ -62,20 +65,20 @@
     <t>IMPELC*,IMPBIO*</t>
   </si>
   <si>
-    <t>*1.5</t>
-  </si>
-  <si>
     <t>~TFM_UPD</t>
   </si>
   <si>
-    <t>*1.375</t>
+    <t>Cset_CN</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0000"/>
+  </numFmts>
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -83,16 +86,40 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color indexed="12"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="43"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -100,12 +127,28 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -121,6 +164,111 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:absoluteUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
+    <sheetNames>
+      <sheetName val="Cover"/>
+      <sheetName val="Regions"/>
+      <sheetName val="config"/>
+      <sheetName val="FF2price"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0"/>
+      <sheetData sheetId="1"/>
+      <sheetData sheetId="2">
+        <row r="3">
+          <cell r="B3">
+            <v>4</v>
+          </cell>
+        </row>
+        <row r="6">
+          <cell r="H6" t="str">
+            <v>Case #</v>
+          </cell>
+          <cell r="I6" t="str">
+            <v>FF_price</v>
+          </cell>
+          <cell r="J6" t="str">
+            <v>ELC, BIO</v>
+          </cell>
+        </row>
+        <row r="7">
+          <cell r="H7">
+            <v>1</v>
+          </cell>
+          <cell r="I7">
+            <v>1.2</v>
+          </cell>
+          <cell r="J7">
+            <v>1.1499999999999999</v>
+          </cell>
+        </row>
+        <row r="8">
+          <cell r="H8">
+            <v>2</v>
+          </cell>
+          <cell r="I8">
+            <v>1.3</v>
+          </cell>
+          <cell r="J8">
+            <v>1.2250000000000001</v>
+          </cell>
+        </row>
+        <row r="9">
+          <cell r="H9">
+            <v>3</v>
+          </cell>
+          <cell r="I9">
+            <v>1.4</v>
+          </cell>
+          <cell r="J9">
+            <v>1.2999999999999998</v>
+          </cell>
+        </row>
+        <row r="10">
+          <cell r="H10">
+            <v>4</v>
+          </cell>
+          <cell r="I10">
+            <v>1.5</v>
+          </cell>
+          <cell r="J10">
+            <v>1.375</v>
+          </cell>
+        </row>
+        <row r="11">
+          <cell r="H11">
+            <v>5</v>
+          </cell>
+          <cell r="I11">
+            <v>1.6</v>
+          </cell>
+          <cell r="J11">
+            <v>1.4500000000000002</v>
+          </cell>
+        </row>
+        <row r="12">
+          <cell r="H12">
+            <v>6</v>
+          </cell>
+          <cell r="I12">
+            <v>2</v>
+          </cell>
+          <cell r="J12">
+            <v>1.75</v>
+          </cell>
+        </row>
+      </sheetData>
+      <sheetData sheetId="3"/>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -386,55 +534,68 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:G5"/>
+  <dimension ref="B7:H15"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="10.33203125" customWidth="1"/>
     <col min="7" max="7" width="15.1328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:7" x14ac:dyDescent="0.45">
-      <c r="B2" t="s">
+    <row r="7" spans="2:8" x14ac:dyDescent="0.45">
+      <c r="B7" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8" spans="2:8" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="B8" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="F8" s="2" t="s">
         <v>9</v>
       </c>
+      <c r="G8" s="3" t="s">
+        <v>5</v>
+      </c>
     </row>
-    <row r="3" spans="2:7" x14ac:dyDescent="0.45">
-      <c r="B3" t="s">
-        <v>0</v>
-      </c>
-      <c r="C3" t="s">
-        <v>1</v>
-      </c>
-      <c r="D3" t="s">
-        <v>2</v>
-      </c>
-      <c r="E3" t="s">
+    <row r="9" spans="2:8" x14ac:dyDescent="0.45">
+      <c r="C9" s="4"/>
+      <c r="D9" t="s">
         <v>4</v>
       </c>
-      <c r="G3" t="s">
-        <v>5</v>
-      </c>
+      <c r="E9" t="str">
+        <f>"*"&amp;VLOOKUP([1]config!$B$3,[1]config!$H$6:$I$12,2,FALSE)</f>
+        <v>*1.5</v>
+      </c>
+      <c r="G9" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="H9" s="5"/>
     </row>
-    <row r="4" spans="2:7" x14ac:dyDescent="0.45">
-      <c r="D4" t="s">
-        <v>3</v>
-      </c>
-      <c r="E4" t="s">
-        <v>8</v>
-      </c>
-      <c r="G4" t="s">
-        <v>6</v>
-      </c>
+    <row r="10" spans="2:8" x14ac:dyDescent="0.45">
+      <c r="D10" t="s">
+        <v>4</v>
+      </c>
+      <c r="E10" t="str">
+        <f>"*"&amp;VLOOKUP([1]config!$B$3,[1]config!$H$6:$J$12,3,FALSE)</f>
+        <v>*1.375</v>
+      </c>
+      <c r="G10" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="H10" s="5"/>
     </row>
-    <row r="5" spans="2:7" x14ac:dyDescent="0.45">
-      <c r="D5" t="s">
-        <v>3</v>
-      </c>
-      <c r="E5" t="s">
-        <v>10</v>
-      </c>
-      <c r="G5" t="s">
-        <v>7</v>
+    <row r="15" spans="2:8" x14ac:dyDescent="0.45">
+      <c r="B15">
+        <v>1000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>